<commit_message>
Complete Phases 1-5: Documentation corrections, Real-time monitoring, AI advisor with Groq, Rule-based risk score, and Test suite
</commit_message>
<xml_diff>
--- a/rpa/input/claims_input.xlsx
+++ b/rpa/input/claims_input.xlsx
@@ -53,156 +53,156 @@
     <t>Meals</t>
   </si>
   <si>
+    <t>2026-10-22</t>
+  </si>
+  <si>
+    <t>Client lunch meeting at Olive Bistro</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_01.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-002</t>
+  </si>
+  <si>
+    <t>2026-10-23</t>
+  </si>
+  <si>
+    <t>Dinner with regional sales team at The Grand</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_02.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-003</t>
+  </si>
+  <si>
+    <t>Priya Patel</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
     <t>2026-10-21</t>
   </si>
   <si>
-    <t>Client lunch meeting at Olive Bistro</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_01.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-002</t>
-  </si>
-  <si>
-    <t>2026-10-22</t>
-  </si>
-  <si>
-    <t>Dinner with regional sales team at The Grand</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_02.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-003</t>
-  </si>
-  <si>
-    <t>Priya Patel</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Travel</t>
+    <t>Airport cab charges to client office</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>CLM-2026-004</t>
+  </si>
+  <si>
+    <t>Office Supplies</t>
+  </si>
+  <si>
+    <t>2026-11-20</t>
+  </si>
+  <si>
+    <t>Wireless keyboard and mouse combo</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_04.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-005</t>
+  </si>
+  <si>
+    <t>Amit Verma</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>2026-10-24</t>
+  </si>
+  <si>
+    <t>Printer ink cartridges and photo paper</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_05.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-006</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>Train tickets for Delhi client deployment</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_06.pdf</t>
+  </si>
+  <si>
+    <t>Train tickets for Delhi client deployment (re-sent)</t>
+  </si>
+  <si>
+    <t>CLM-2026-007</t>
+  </si>
+  <si>
+    <t>2026-12-05</t>
+  </si>
+  <si>
+    <t>Annual team celebration dinner</t>
+  </si>
+  <si>
+    <t>CLM-2026-008</t>
+  </si>
+  <si>
+    <t>Accommodation</t>
+  </si>
+  <si>
+    <t>2026-10-15</t>
+  </si>
+  <si>
+    <t>2 nights stay at Lemon Tree Premier for tech conference</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_08.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-009</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>Luxury suite hotel stay during offsite</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_09.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-010</t>
+  </si>
+  <si>
+    <t>Client Entertainment</t>
   </si>
   <si>
     <t>2026-10-20</t>
   </si>
   <si>
-    <t>Airport cab charges to client office</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>CLM-2026-004</t>
-  </si>
-  <si>
-    <t>Office Supplies</t>
-  </si>
-  <si>
-    <t>2026-11-19</t>
-  </si>
-  <si>
-    <t>Wireless keyboard and mouse combo</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_04.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-005</t>
-  </si>
-  <si>
-    <t>Amit Verma</t>
-  </si>
-  <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>2026-10-23</t>
-  </si>
-  <si>
-    <t>Printer ink cartridges and photo paper</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_05.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-006</t>
-  </si>
-  <si>
-    <t>2026-10-17</t>
-  </si>
-  <si>
-    <t>Train tickets for Delhi client deployment</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_06.pdf</t>
-  </si>
-  <si>
-    <t>Train tickets for Delhi client deployment (re-sent)</t>
-  </si>
-  <si>
-    <t>CLM-2026-007</t>
-  </si>
-  <si>
-    <t>2026-12-04</t>
-  </si>
-  <si>
-    <t>Annual team celebration dinner</t>
-  </si>
-  <si>
-    <t>CLM-2026-008</t>
-  </si>
-  <si>
-    <t>Accommodation</t>
+    <t>Coffee and snacks with prospective vendor partners</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_10.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-011</t>
+  </si>
+  <si>
+    <t>Certifications</t>
   </si>
   <si>
     <t>2026-10-14</t>
   </si>
   <si>
-    <t>2 nights stay at Lemon Tree Premier for tech conference</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_08.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-009</t>
-  </si>
-  <si>
-    <t>2026-10-18</t>
-  </si>
-  <si>
-    <t>Luxury suite hotel stay during offsite</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_09.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-010</t>
-  </si>
-  <si>
-    <t>Client Entertainment</t>
-  </si>
-  <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>Coffee and snacks with prospective vendor partners</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_10.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-011</t>
-  </si>
-  <si>
-    <t>Certifications</t>
-  </si>
-  <si>
-    <t>2026-10-13</t>
-  </si>
-  <si>
     <t>AWS Certified Solutions Architect exam fee</t>
   </si>
   <si>
@@ -212,7 +212,7 @@
     <t>CLM-2026-012</t>
   </si>
   <si>
-    <t>2026-10-24</t>
+    <t>2026-10-25</t>
   </si>
   <si>
     <t>Whiteboard markers and sticky notes for brainstorming</t>
@@ -242,7 +242,7 @@
     <t>CLM-2026-015</t>
   </si>
   <si>
-    <t>2026-10-25</t>
+    <t>2026-10-26</t>
   </si>
   <si>
     <t>Uber rides for client product presentation</t>

</xml_diff>

<commit_message>
docs: align all documentation, reports, and viva guide with 7/5/4 benchmark breakdown and rejection rules
</commit_message>
<xml_diff>
--- a/rpa/input/claims_input.xlsx
+++ b/rpa/input/claims_input.xlsx
@@ -53,196 +53,196 @@
     <t>Meals</t>
   </si>
   <si>
+    <t>2026-10-21</t>
+  </si>
+  <si>
+    <t>Client lunch meeting at Olive Bistro</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_01.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-002</t>
+  </si>
+  <si>
     <t>2026-10-22</t>
   </si>
   <si>
-    <t>Client lunch meeting at Olive Bistro</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_01.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-002</t>
+    <t>Dinner with regional sales team at The Grand</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_02.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-003</t>
+  </si>
+  <si>
+    <t>Priya Patel</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>2026-10-20</t>
+  </si>
+  <si>
+    <t>Airport cab charges to client office</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>CLM-2026-004</t>
+  </si>
+  <si>
+    <t>Office Supplies</t>
+  </si>
+  <si>
+    <t>2026-11-19</t>
+  </si>
+  <si>
+    <t>Wireless keyboard and mouse combo</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_04.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-005</t>
+  </si>
+  <si>
+    <t>Amit Verma</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
   </si>
   <si>
     <t>2026-10-23</t>
   </si>
   <si>
-    <t>Dinner with regional sales team at The Grand</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_02.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-003</t>
-  </si>
-  <si>
-    <t>Priya Patel</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Travel</t>
-  </si>
-  <si>
-    <t>2026-10-21</t>
-  </si>
-  <si>
-    <t>Airport cab charges to client office</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>CLM-2026-004</t>
-  </si>
-  <si>
-    <t>Office Supplies</t>
-  </si>
-  <si>
-    <t>2026-11-20</t>
-  </si>
-  <si>
-    <t>Wireless keyboard and mouse combo</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_04.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-005</t>
-  </si>
-  <si>
-    <t>Amit Verma</t>
-  </si>
-  <si>
-    <t>Human Resources</t>
+    <t>Printer ink cartridges and photo paper</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_05.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-006</t>
+  </si>
+  <si>
+    <t>2026-10-17</t>
+  </si>
+  <si>
+    <t>Train tickets for Delhi client deployment</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_06.pdf</t>
+  </si>
+  <si>
+    <t>Train tickets for Delhi client deployment (re-sent)</t>
+  </si>
+  <si>
+    <t>CLM-2026-007</t>
+  </si>
+  <si>
+    <t>2026-12-04</t>
+  </si>
+  <si>
+    <t>Annual team celebration dinner</t>
+  </si>
+  <si>
+    <t>CLM-2026-008</t>
+  </si>
+  <si>
+    <t>Accommodation</t>
+  </si>
+  <si>
+    <t>2026-10-14</t>
+  </si>
+  <si>
+    <t>2 nights stay at Lemon Tree Premier for tech conference</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_08.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-009</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>Luxury suite hotel stay during offsite</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_09.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-010</t>
+  </si>
+  <si>
+    <t>Client Entertainment</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>Coffee and snacks with prospective vendor partners</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_10.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-011</t>
+  </si>
+  <si>
+    <t>Certifications</t>
+  </si>
+  <si>
+    <t>2026-10-13</t>
+  </si>
+  <si>
+    <t>AWS Certified Solutions Architect exam fee</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_11.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-012</t>
   </si>
   <si>
     <t>2026-10-24</t>
   </si>
   <si>
-    <t>Printer ink cartridges and photo paper</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_05.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-006</t>
-  </si>
-  <si>
-    <t>2026-10-18</t>
-  </si>
-  <si>
-    <t>Train tickets for Delhi client deployment</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_06.pdf</t>
-  </si>
-  <si>
-    <t>Train tickets for Delhi client deployment (re-sent)</t>
-  </si>
-  <si>
-    <t>CLM-2026-007</t>
-  </si>
-  <si>
-    <t>2026-12-05</t>
-  </si>
-  <si>
-    <t>Annual team celebration dinner</t>
-  </si>
-  <si>
-    <t>CLM-2026-008</t>
-  </si>
-  <si>
-    <t>Accommodation</t>
-  </si>
-  <si>
-    <t>2026-10-15</t>
-  </si>
-  <si>
-    <t>2 nights stay at Lemon Tree Premier for tech conference</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_08.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-009</t>
-  </si>
-  <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>Luxury suite hotel stay during offsite</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_09.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-010</t>
-  </si>
-  <si>
-    <t>Client Entertainment</t>
-  </si>
-  <si>
-    <t>2026-10-20</t>
-  </si>
-  <si>
-    <t>Coffee and snacks with prospective vendor partners</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_10.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-011</t>
-  </si>
-  <si>
-    <t>Certifications</t>
-  </si>
-  <si>
-    <t>2026-10-14</t>
-  </si>
-  <si>
-    <t>AWS Certified Solutions Architect exam fee</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_11.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-012</t>
+    <t>Whiteboard markers and sticky notes for brainstorming</t>
+  </si>
+  <si>
+    <t>CLM-2026-013</t>
+  </si>
+  <si>
+    <t>Gym Membership</t>
+  </si>
+  <si>
+    <t>Monthly fitness center wellness reimbursement</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_14.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-014</t>
+  </si>
+  <si>
+    <t>Project delivery team dinner at Barbeque Nation</t>
+  </si>
+  <si>
+    <t>uploads/receipts/sample_receipt_15.pdf</t>
+  </si>
+  <si>
+    <t>CLM-2026-015</t>
   </si>
   <si>
     <t>2026-10-25</t>
-  </si>
-  <si>
-    <t>Whiteboard markers and sticky notes for brainstorming</t>
-  </si>
-  <si>
-    <t>CLM-2026-013</t>
-  </si>
-  <si>
-    <t>Gym Membership</t>
-  </si>
-  <si>
-    <t>Monthly fitness center wellness reimbursement</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_14.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-014</t>
-  </si>
-  <si>
-    <t>Project delivery team dinner at Barbeque Nation</t>
-  </si>
-  <si>
-    <t>uploads/receipts/sample_receipt_15.pdf</t>
-  </si>
-  <si>
-    <t>CLM-2026-015</t>
-  </si>
-  <si>
-    <t>2026-10-26</t>
   </si>
   <si>
     <t>Uber rides for client product presentation</t>

</xml_diff>